<commit_message>
updates reflecting V1 of the PCB
</commit_message>
<xml_diff>
--- a/electronics/KiCad/1_Distribution_Board/bom/1_Distribution Board_JLPCB_BOM.xlsx
+++ b/electronics/KiCad/1_Distribution_Board/bom/1_Distribution Board_JLPCB_BOM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EfFr3ek\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EfFr3ek\Documents\GitHub\sorter-v2\electronics\KiCad\1_Distribution_Board\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{0E9B7734-0033-46AB-A78F-F088742743E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A386231-BFB9-442C-9153-00C99EDEB618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{241FB4BB-BF10-472E-B5E2-02B5DA3EADB7}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{241FB4BB-BF10-472E-B5E2-02B5DA3EADB7}"/>
   </bookViews>
   <sheets>
     <sheet name="1_Distribution Board" sheetId="1" r:id="rId1"/>
@@ -675,7 +675,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -853,6 +853,18 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1016,8 +1028,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1450,7 +1464,7 @@
       <c r="D2" t="s">
         <v>78</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="1">
         <v>6</v>
       </c>
       <c r="F2" t="s">
@@ -1473,7 +1487,7 @@
       <c r="D3" t="s">
         <v>79</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="1">
         <v>6</v>
       </c>
       <c r="F3" t="s">
@@ -1496,7 +1510,7 @@
       <c r="D4" t="s">
         <v>85</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="1">
         <v>4</v>
       </c>
       <c r="F4" t="s">
@@ -1522,7 +1536,7 @@
       <c r="D5" t="s">
         <v>88</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="1">
         <v>35</v>
       </c>
       <c r="F5" t="s">
@@ -1545,7 +1559,7 @@
       <c r="D6" t="s">
         <v>89</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="1">
         <v>4</v>
       </c>
       <c r="F6" t="s">
@@ -1568,7 +1582,7 @@
       <c r="D7" t="s">
         <v>92</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="1">
         <v>2</v>
       </c>
       <c r="F7" t="s">
@@ -1591,7 +1605,7 @@
       <c r="D8" t="s">
         <v>94</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="1">
         <v>1</v>
       </c>
       <c r="F8" t="s">
@@ -1614,7 +1628,7 @@
       <c r="D9" t="s">
         <v>95</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="1">
         <v>1</v>
       </c>
       <c r="F9" t="s">
@@ -1637,7 +1651,7 @@
       <c r="D10" t="s">
         <v>161</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="1">
         <v>1</v>
       </c>
       <c r="F10" t="s">
@@ -1756,7 +1770,7 @@
       <c r="D14" t="s">
         <v>144</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="1">
         <v>2</v>
       </c>
       <c r="F14" t="s">
@@ -1779,7 +1793,7 @@
       <c r="D15" t="s">
         <v>163</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="1">
         <v>2</v>
       </c>
       <c r="F15" t="s">
@@ -1802,7 +1816,7 @@
       <c r="D16" t="s">
         <v>141</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="1">
         <v>1</v>
       </c>
       <c r="F16" t="s">
@@ -1825,7 +1839,7 @@
       <c r="D17" t="s">
         <v>167</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="1">
         <v>1</v>
       </c>
       <c r="F17" t="s">
@@ -1848,7 +1862,7 @@
       <c r="D18" t="s">
         <v>136</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="1">
         <v>4</v>
       </c>
       <c r="F18" t="s">
@@ -1871,7 +1885,7 @@
       <c r="D19" t="s">
         <v>165</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="1">
         <v>2</v>
       </c>
       <c r="F19" t="s">
@@ -1894,7 +1908,7 @@
       <c r="D20" t="s">
         <v>159</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="1">
         <v>1</v>
       </c>
       <c r="F20" t="s">
@@ -1917,7 +1931,7 @@
       <c r="D21" t="s">
         <v>126</v>
       </c>
-      <c r="E21">
+      <c r="E21" s="1">
         <v>12</v>
       </c>
       <c r="F21" t="s">
@@ -1940,7 +1954,7 @@
       <c r="D22" t="s">
         <v>120</v>
       </c>
-      <c r="E22">
+      <c r="E22" s="1">
         <v>4</v>
       </c>
       <c r="F22" t="s">
@@ -1963,7 +1977,7 @@
       <c r="D23" t="s">
         <v>107</v>
       </c>
-      <c r="E23">
+      <c r="E23" s="1">
         <v>4</v>
       </c>
       <c r="F23" t="s">
@@ -1986,7 +2000,7 @@
       <c r="D24" t="s">
         <v>130</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="1">
         <v>4</v>
       </c>
       <c r="F24" t="s">
@@ -2009,7 +2023,7 @@
       <c r="D25" t="s">
         <v>100</v>
       </c>
-      <c r="E25">
+      <c r="E25" s="1">
         <v>6</v>
       </c>
       <c r="F25" t="s">
@@ -2032,7 +2046,7 @@
       <c r="D26" t="s">
         <v>102</v>
       </c>
-      <c r="E26">
+      <c r="E26" s="1">
         <v>12</v>
       </c>
       <c r="F26" t="s">
@@ -2055,7 +2069,7 @@
       <c r="D27" t="s">
         <v>119</v>
       </c>
-      <c r="E27">
+      <c r="E27" s="2">
         <v>3</v>
       </c>
       <c r="F27" t="s">
@@ -2078,7 +2092,7 @@
       <c r="D28" t="s">
         <v>123</v>
       </c>
-      <c r="E28">
+      <c r="E28" s="1">
         <v>1</v>
       </c>
       <c r="F28" t="s">
@@ -2101,7 +2115,7 @@
       <c r="D29" t="s">
         <v>125</v>
       </c>
-      <c r="E29">
+      <c r="E29" s="1">
         <v>1</v>
       </c>
       <c r="F29" t="s">
@@ -2124,7 +2138,7 @@
       <c r="D30" t="s">
         <v>115</v>
       </c>
-      <c r="E30">
+      <c r="E30" s="1">
         <v>1</v>
       </c>
       <c r="F30" t="s">
@@ -2147,7 +2161,7 @@
       <c r="D31" t="s">
         <v>132</v>
       </c>
-      <c r="E31">
+      <c r="E31" s="1">
         <v>4</v>
       </c>
       <c r="F31" t="s">
@@ -2170,7 +2184,7 @@
       <c r="D32" t="s">
         <v>135</v>
       </c>
-      <c r="E32">
+      <c r="E32" s="1">
         <v>2</v>
       </c>
       <c r="F32" t="s">
@@ -2193,7 +2207,7 @@
       <c r="D33" t="s">
         <v>139</v>
       </c>
-      <c r="E33">
+      <c r="E33" s="1">
         <v>1</v>
       </c>
       <c r="F33" t="s">

</xml_diff>